<commit_message>
feat(F-NAR-019): ATOM-DIF.PAR.001-04 La pièce du puzzle
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.PAR.001-04.xlsx
+++ b/stories/arbres/ATOM-DIF.PAR.001-04.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le bateau sur le rebord</t>
+          <t>La pièce du puzzle</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>classe au bac d'eau, puis parc</t>
+          <t>école : classe, crayon jaune sous la table, craie, vitre, cartable, puzzle d'animaux ; puis parc</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut faire flotter son bateau en papier dans le bac d'eau. Victorina parle peu. Il lui tend le bateau. Plus tard au parc, ils font un port de sable. Le bateau a un quai.</t>
+          <t>Un crayon jaune roule sous la table. Sur le bord, un éclat de table brille. Amir veut finir le puzzle, maintenant. Victorina parle peu. Il pousse trop vite : la pièce tombe. Sourire parti, poitrine, papa accroupi. Il refuse de foncer, tend la pièce, attend. 2e ruse au parc. Merci vécu. Un éclat de table tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un bateau en papier sèche sur le rebord. Une goutte a marqué la proue. Le papier sent encore la colle. Le pliage est un peu raide. Une fenêtre est entrouverte. L'air sent la craie. Papa range le cartable d'Amir. Maman glisse une pomme dans la poche. La pomme est lisse et froide. Tu as vu la goutte, Amir ? Elle a fait une tache. Je te dis au revoir ici. Papa t'attend au parc, plus tard. En ce moment, Amir prend le bateau. Le bac d'eau brille près de la fenêtre. L'eau est claire et froide. Je veux qu'il flotte. Jusqu'à l'autre bord. Tout droit, alors. Victorina est déjà là. Victorina parle peu. Elle regarde ses chaussures. Les lacets sont verts. Amir a envie de poser beaucoup de questions. Il respire. On peut attendre. Tu peux tendre un jouet. Le bateau est léger dans sa main. Victorina ne dit rien.</t>
+          <t>Un toc sec court sous le bois. Un crayon jaune file, puis s'arrête. Il roule, papa ! Il est passé sous la table ? Oui, papa. Papa se penche près du pied. L'air de la classe sent la craie. Ça sent la craie, maman. Tu le sens, toi ? Oui, maman. Une vitre laisse un carré de soleil. Tu vois le carré, Amir ? Oui, sur le bois. Le cartable penche contre une jambe. Le cartable tient tout seul ? Oui, maman. Sur le bord, un éclat de table brille. Il brille, papa ! Tu le vois, ce petit point ? Oui, un petit point. Un puzzle d'animaux attend sur le bois. Le chat n'a pas de tête. Il manque une pièce, Amir ? Oui, la tête. En ce moment, Amir veut finir le puzzle. Je veux le finir, maintenant ! Toute la tête, maman. Avec Victorina, Amir ? Oui, papa. Victorina s'assoit près de la table. Victorina parle peu. Elle regarde ses mains. Victorina ! Amir ouvre la bouche trop vite. Les questions montent, serrées. Il pousse la tête du chat. La tête, vite ! La pièce glisse trop fort. Elle tombe sous la table. Oh ! Elle rejoint le crayon jaune. Elle est tombée ! Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu, lourdes. Papa s'accroupit à la même hauteur. Tu veux le chat avec Victorina ? Oui, papa. Tes mains sont serrées, Amir ? Un peu, maman. Amir refuse de foncer. Il ramasse la pièce, sans se presser. Le crayon jaune reste sous le bois. Personne ne parle. Il observe le bord, un instant. L'éclat de table tremble, puis tient. L'éclat, papa ? Tu le vois, toi ? Oui, sur le bois. Amir tend la pièce, la main ouverte. Victorina ne dit rien.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un bateau en papier sèche sur le rebord. Une goutte a marqué la proue. Le papier sent encore la colle. Le pliage est un peu raide. Une fenêtre est entrouverte. L'air sent la craie. Papa range le cartable d'Amir. Maman glisse une pomme dans la poche. La pomme est lisse et froide. Tu as vu la goutte, Amir ? Elle a fait une tache. Je te dis au revoir ici. Papa t'attend au parc, plus tard. En ce moment, Amir prend le bateau. Le bac d'eau brille près de la fenêtre. L'eau est claire et froide. Je veux qu'il flotte. Jusqu'à l'autre bord. Tout droit, alors. Victorina est déjà là. Victorina parle peu. Elle regarde ses chaussures. Les lacets sont verts. Amir a envie de poser beaucoup de questions. Il respire. On peut attendre. Tu peux tendre un jouet. Le bateau est léger dans sa main. Victorina ne dit rien.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un toc sec court sous le bois. Un crayon jaune file, puis s'arrête. Il roule, papa ! Il est passé sous la table ? Oui, papa. Papa se penche près du pied. L'air de la classe sent la craie. Ça sent la craie, maman. Tu le sens, toi ? Oui, maman. Une vitre laisse un carré de soleil. Tu vois le carré, Amir ? Oui, sur le bois. Le cartable penche contre une jambe. Le cartable tient tout seul ? Oui, maman. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de table&lt;/emphasis&gt; brille. Il brille, papa ! Tu le vois, ce petit point ? Oui, un petit point. Un puzzle d'animaux attend sur le bois. Le chat n'a pas de tête. Il manque une pièce, Amir ? Oui, la tête. En ce moment, Amir veut finir le puzzle. Je veux le finir, maintenant ! Toute la tête, maman. Avec Victorina, Amir ? Oui, papa. Victorina s'assoit près de la table. Victorina parle peu. Elle regarde ses mains. Victorina ! Amir ouvre la bouche trop vite. Les questions montent, serrées. Il pousse la tête du chat. La tête, vite ! La pièce glisse trop fort. Elle tombe sous la table. Oh ! Elle rejoint le crayon jaune. Elle est tombée ! Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu, lourdes. Papa s'accroupit à la même hauteur. Tu veux le chat avec Victorina ? Oui, papa. Tes mains sont serrées, Amir ? Un peu, maman. Amir refuse de foncer. Il ramasse la pièce, sans se presser. Le crayon jaune reste sous le bois. Personne ne parle. Il observe le bord, un instant. L'éclat de table tremble, puis tient. L'éclat, papa ? Tu le vois, toi ? Oui, sur le bois. Amir tend la pièce, la main ouverte. Victorina ne dit rien.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Ruben arrive en classe avec maman. Maman dit au revoir. Iris est déjà là. Iris parle peu. Elle regarde ses chaussures. Ruben veut poser beaucoup de questions. Il ouvre la bouche. La maîtresse dit doucement : on peut &lt;emphasis&gt;attendre&lt;/emphasis&gt;. On n'imite pas. On ne va pas forcer la parole. Ruben ferme la bouche. Il respire. Il prend un puzzle d'animaux. Il va tendre un jouet. Il tend une pièce vers Iris. Iris regarde. Elle ne dit rien. Ruben attend. La classe est calme. On entend un oiseau dehors. Iris prend la pièce. Elle la pose. Ruben sourit. Plus tard, au parc, maman est au banc. Iris est là aussi. Elle parle peu. Ruben prend un seau. Il va tendre un jouet. Il tend le seau. Iris le prend. Elle remplit le seau de sable. Ruben attend. Iris ne parle toujours pas. C'est possible. Maman dit : on peut attendre. On peut tendre un jouet. On ne va pas forcer la parole. Ruben hoche la tête. Ils font un tas de sable. Un silence. Puis Iris dit tout bas : sable. Ruben dit : sable. Ils jouent. Le jeu a eu lieu, même avec peu de mots. [pause]</t>
+          <t>Un toc sec court sous le bois. Un crayon jaune file, puis s'arrête. Il roule, papa ! Il est passé sous la table ? Oui, papa. Papa se penche près du pied. L'air de la classe sent la craie. Ça sent la craie, maman. Tu le sens, toi ? Oui, maman. Une vitre laisse un carré de soleil. Tu vois le carré, Amir ? Oui, sur le bois. Le cartable penche contre une jambe. Le cartable tient tout seul ? Oui, maman. Sur le bord, un &lt;emphasis&gt;éclat de table&lt;/emphasis&gt; brille. Il brille, papa ! Tu le vois, ce petit point ? Oui, un petit point. Un puzzle d'animaux attend sur le bois. Le chat n'a pas de tête. Il manque une pièce, Amir ? Oui, la tête. En ce moment, Amir veut finir le puzzle. Je veux le finir, maintenant ! Toute la tête, maman. Avec Victorina, Amir ? Oui, papa. Victorina s'assoit près de la table. Victorina parle peu. Elle regarde ses mains. Victorina ! Amir ouvre la bouche trop vite. Les questions montent, serrées. Il pousse la tête du chat. La tête, vite ! La pièce glisse trop fort. Elle tombe sous la table. Oh ! Elle rejoint le crayon jaune. Elle est tombée ! Le sourire d'Amir disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu, lourdes. Papa s'accroupit à la même hauteur. Tu veux le chat avec Victorina ? Oui, papa. Tes mains sont serrées, Amir ? Un peu, maman. Amir refuse de foncer. Il ramasse la pièce, sans se presser. Le crayon jaune reste sous le bois. Personne ne parle. Il observe le bord, un instant. L'éclat de table tremble, puis tient. L'éclat, papa ? Tu le vois, toi ? Oui, sur le bois. Amir tend la pièce, la main ouverte. Victorina ne dit rien. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>éclat de table</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,43 +1326,79 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_finir_le_puzzle_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un bateau en papier sèche sur le rebord.
-narrateur|Une goutte a marqué la proue.
-narrateur|Le papier sent encore la colle.
-narrateur|Le pliage est un peu raide.
-narrateur|Une fenêtre est entrouverte.
-narrateur|L'air sent la craie.
-narrateur|Papa range le cartable d'Amir.
-narrateur|Maman glisse une pomme dans la poche.
-narrateur|La pomme est lisse et froide.
-papa|Tu as vu la goutte, Amir ?
-enfant-m|Elle a fait une tache.
-maman|Je te dis au revoir ici.
-maman|Papa t'attend au parc, plus tard.
-narrateur|En ce moment, Amir prend le bateau.
-narrateur|Le bac d'eau brille près de la fenêtre.
-narrateur|L'eau est claire et froide.
-enfant-m|Je veux qu'il flotte.
-enfant-m|Jusqu'à l'autre bord.
-papa|Tout droit, alors.
-narrateur|Victorina est déjà là.
+          <t>narrateur|Un toc sec court sous le bois.
+narrateur|Un crayon jaune file, puis s'arrête.
+enfant-m|Il roule, papa !
+papa|Il est passé sous la table ?
+enfant-m|Oui, papa.
+narrateur|Papa se penche près du pied.
+narrateur|L'air de la classe sent la craie.
+enfant-m|Ça sent la craie, maman.
+maman|Tu le sens, toi ?
+enfant-m|Oui, maman.
+narrateur|Une vitre laisse un carré de soleil.
+papa|Tu vois le carré, Amir ?
+enfant-m|Oui, sur le bois.
+narrateur|Le cartable penche contre une jambe.
+maman|Le cartable tient tout seul ?
+enfant-m|Oui, maman.
+narrateur|Sur le bord, un éclat de table brille.
+enfant-m|Il brille, papa !
+papa|Tu le vois, ce petit point ?
+enfant-m|Oui, un petit point.
+narrateur|Un puzzle d'animaux attend sur le bois.
+enfant-m|Le chat n'a pas de tête.
+maman|Il manque une pièce, Amir ?
+enfant-m|Oui, la tête.
+narrateur|En ce moment, Amir veut finir le puzzle.
+enfant-m|Je veux le finir, maintenant !
+enfant-m|Toute la tête, maman.
+papa|Avec Victorina, Amir ?
+enfant-m|Oui, papa.
+narrateur|Victorina s'assoit près de la table.
 narrateur|Victorina parle peu.
-narrateur|Elle regarde ses chaussures.
-narrateur|Les lacets sont verts.
-narrateur|Amir a envie de poser beaucoup de questions.
-narrateur|Il respire.
-maman|On peut attendre.
-papa|Tu peux tendre un jouet.
-narrateur|Le bateau est léger dans sa main.
+narrateur|Elle regarde ses mains.
+enfant-m|Victorina !
+narrateur|Amir ouvre la bouche trop vite.
+narrateur|Les questions montent, serrées.
+narrateur|Il pousse la tête du chat.
+enfant-m|La tête, vite !
+narrateur|La pièce glisse trop fort.
+narrateur|Elle tombe sous la table.
+enfant-m|Oh !
+narrateur|Elle rejoint le crayon jaune.
+enfant-m|Elle est tombée !
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu, lourdes.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu veux le chat avec Victorina ?
+enfant-m|Oui, papa.
+maman|Tes mains sont serrées, Amir ?
+enfant-m|Un peu, maman.
+narrateur|Amir refuse de foncer.
+narrateur|Il ramasse la pièce, sans se presser.
+narrateur|Le crayon jaune reste sous le bois.
+narrateur|Personne ne parle.
+narrateur|Il observe le bord, un instant.
+narrateur|L'éclat de table tremble, puis tient.
+enfant-m|L'éclat, papa ?
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur le bois.
+narrateur|Amir tend la pièce, la main ouverte.
 narrateur|Victorina ne dit rien.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>crayon,craie</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1430,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorina parle peu. Que fait Amir ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorina parle &lt;emphasis level="moderate"&gt;peu&lt;/emphasis&gt;. Que fait Amir ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Iris parle peu. Que fait Ruben ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorina parle &lt;emphasis&gt;peu&lt;/emphasis&gt;. Que fait Amir ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1409,7 +1445,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>attendre | tendre un jouet | un jouet | le bateau | il attend</t>
+          <t>attendre | tendre un jouet | un jouet | il attend</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1462,7 +1498,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1470,10 +1506,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1488,34 +1524,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>peu</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1524,23 +1564,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=victorina_parle_peu_que_fait_amir; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1573,17 +1613,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir tend le bateau. Pour toi. Il attend. Une feuille tape encore la vitre. Victorina prend le bateau. Elle le pose sur l'eau. Le papier avance tout doux. On ne force pas la parole. Le bateau n'a pas besoin de mots. Amir souffle un peu. Une petite vague va jusqu'au bord. Le bateau touche l'autre bord. Le papier est un peu mouillé. Il est arrivé. Victorina dit tout bas. Bateau. Bateau. Tu as su attendre. Bravo, Amir. Plus tard, au parc, papa est au banc. Maman arrive avec le goûter. Le sac sent la pomme. Victorina est là aussi. Amir tend un seau. Le seau est tiède. Victorina le remplit de sable. Ils font un port, tout bas. Le sable est frais sous les doigts. Un quai. Une crique. Un trou d'eau. Port. Port.</t>
+          <t>Amir tend la pièce, sans se presser. Pour toi. Sa main reste ouverte. Il attend. Victorina regarde la pièce. Elle ne parle pas. Elle prend la pièce, sans bruit. Elle pose la tête du chat. Le chat, papa. Tu le vois, le chat ? Oui, papa. Chat. Chat. Le museau est gris, Amir ? Oui, maman. Amir veut demander le chien. Il referme un peu la bouche. Il glisse une autre pièce, plus lente. C'est le dos, Amir ? Le dos du chien. Victorina pose sa main à côté. Elle reste les mains sur le bois. À toi. Elle pose une oreille. Chien. Chien. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. Le puzzle avance, vous deux ? Oui, papa. Tes doigts sont moins serrés, Amir ? Oui, maman. Il observe l'éclat de table. Le point, papa. Sur le bois, Amir ? Oui, il tient. On met le puzzle dans le cartable ? Oui, maman. Le crayon jaune reste sous la table. Il reste là. On le laisse, Amir ? Oui, papa.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir tend le bateau. Pour toi. Il attend. Une feuille tape encore la vitre. Victorina prend le bateau. Elle le pose sur l'eau. Le papier avance tout doux. On ne force pas la parole. Le bateau n'a pas besoin de mots. Amir souffle un peu. Une petite vague va jusqu'au bord. Le bateau touche l'autre bord. Le papier est un peu mouillé. Il est arrivé. Victorina dit tout bas. Bateau. Bateau. Tu as su attendre. Bravo, Amir. Plus tard, au parc, papa est au banc. Maman arrive avec le goûter. Le sac sent la pomme. Victorina est là aussi. Amir tend un seau. Le seau est tiède. Victorina le remplit de sable. Ils font un port, tout bas. Le sable est frais sous les doigts. Un quai. Une crique. Un trou d'eau. Port. Port.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir tend la &lt;emphasis level="moderate"&gt;pièce&lt;/emphasis&gt;, sans se presser. Pour toi. Sa main reste ouverte. Il attend. Victorina regarde la pièce. Elle ne parle pas. Elle prend la pièce, sans bruit. Elle pose la tête du chat. Le chat, papa. Tu le vois, le chat ? Oui, papa. Chat. Chat. Le museau est gris, Amir ? Oui, maman. Amir veut demander le chien. Il referme un peu la bouche. Il glisse une autre pièce, plus lente. C'est le dos, Amir ? Le dos du chien. Victorina pose sa main à côté. Elle reste les mains sur le bois. À toi. Elle pose une oreille. Chien. Chien. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. Le puzzle avance, vous deux ? Oui, papa. Tes doigts sont moins serrés, Amir ? Oui, maman. Il observe l'éclat de table. Le point, papa. Sur le bois, Amir ? Oui, il tient. On met le puzzle dans le cartable ? Oui, maman. Le crayon jaune reste sous la table. Il reste là. On le laisse, Amir ? Oui, papa.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Ruben a su &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Il a tendu un jouet. Iris a pris le seau. On n'a pas forcé la parole. [pause]</t>
+          <t>Amir tend la &lt;emphasis&gt;pièce&lt;/emphasis&gt;, sans se presser. Pour toi. Sa main reste ouverte. Il attend. Victorina regarde la pièce. Elle ne parle pas. Elle prend la pièce, sans bruit. Elle pose la tête du chat. Le chat, papa. Tu le vois, le chat ? Oui, papa. Chat. Chat. Le museau est gris, Amir ? Oui, maman. Amir veut demander le chien. Il referme un peu la bouche. Il glisse une autre pièce, plus lente. C'est le dos, Amir ? Le dos du chien. Victorina pose sa main à côté. Elle reste les mains sur le bois. À toi. Elle pose une oreille. Chien. Chien. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. Le puzzle avance, vous deux ? Oui, papa. Tes doigts sont moins serrés, Amir ? Oui, maman. Il observe l'éclat de table. Le point, papa. Sur le bois, Amir ? Oui, il tient. On met le puzzle dans le cartable ? Oui, maman. Le crayon jaune reste sous la table. Il reste là. On le laisse, Amir ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1630,7 +1670,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1638,10 +1678,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1664,30 +1704,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>pièce</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1696,10 +1736,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1712,49 +1752,58 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_tend_la_piece_il_attend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir tend le bateau.
+          <t>narrateur|Amir tend la pièce, sans se presser.
 enfant-m|Pour toi.
+narrateur|Sa main reste ouverte.
 narrateur|Il attend.
-narrateur|Une feuille tape encore la vitre.
-narrateur|Victorina prend le bateau.
-narrateur|Elle le pose sur l'eau.
-narrateur|Le papier avance tout doux.
-maman|On ne force pas la parole.
-papa|Le bateau n'a pas besoin de mots.
-narrateur|Amir souffle un peu.
-narrateur|Une petite vague va jusqu'au bord.
-narrateur|Le bateau touche l'autre bord.
-narrateur|Le papier est un peu mouillé.
-enfant-m|Il est arrivé.
-narrateur|Victorina dit tout bas.
-enfant-f|Bateau.
-enfant-m|Bateau.
-papa|Tu as su attendre.
-papa|Bravo, Amir.
-narrateur|Plus tard, au parc, papa est au banc.
-narrateur|Maman arrive avec le goûter.
-narrateur|Le sac sent la pomme.
-narrateur|Victorina est là aussi.
-narrateur|Amir tend un seau.
-narrateur|Le seau est tiède.
-narrateur|Victorina le remplit de sable.
-narrateur|Ils font un port, tout bas.
-narrateur|Le sable est frais sous les doigts.
-narrateur|Un quai.
-narrateur|Une crique.
-narrateur|Un trou d'eau.
-enfant-f|Port.
-enfant-m|Port.</t>
+narrateur|Victorina regarde la pièce.
+narrateur|Elle ne parle pas.
+narrateur|Elle prend la pièce, sans bruit.
+narrateur|Elle pose la tête du chat.
+enfant-m|Le chat, papa.
+papa|Tu le vois, le chat ?
+enfant-m|Oui, papa.
+copine|Chat.
+enfant-m|Chat.
+maman|Le museau est gris, Amir ?
+enfant-m|Oui, maman.
+narrateur|Amir veut demander le chien.
+narrateur|Il referme un peu la bouche.
+narrateur|Il glisse une autre pièce, plus lente.
+papa|C'est le dos, Amir ?
+enfant-m|Le dos du chien.
+narrateur|Victorina pose sa main à côté.
+narrateur|Elle reste les mains sur le bois.
+enfant-m|À toi.
+narrateur|Elle pose une oreille.
+copine|Chien.
+enfant-m|Chien.
+narrateur|Le ventre d'Amir se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|Le puzzle avance, vous deux ?
+enfant-m|Oui, papa.
+maman|Tes doigts sont moins serrés, Amir ?
+enfant-m|Oui, maman.
+narrateur|Il observe l'éclat de table.
+enfant-m|Le point, papa.
+papa|Sur le bois, Amir ?
+enfant-m|Oui, il tient.
+maman|On met le puzzle dans le cartable ?
+enfant-m|Oui, maman.
+narrateur|Le crayon jaune reste sous la table.
+enfant-m|Il reste là.
+papa|On le laisse, Amir ?
+enfant-m|Oui, papa.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>puzzle,craie</t>
         </is>
       </c>
     </row>
@@ -1781,17 +1830,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman aide Victorina à mettre son manteau. Les boutons sont ronds et lisses. Victorina fait un petit signe. À demain ? À demain. Le bateau sèche encore sur le rebord. Et le port reste au parc. Deux eaux, aujourd'hui. La pomme reste dans la poche. Le bateau sèche encore un peu. La tache est partie.</t>
+          <t>Au parc, une table de bois se tient près de l'herbe. Tu poses le puzzle ici, Amir ? Oui, papa. Maman ouvre le cartable sur l'herbe. Le chat est entier, Amir ? Le chien n'est pas fini. Victorina s'assoit, sans un mot. Je finis, maintenant ! Il pousse la dernière pièce trop vite. La pièce part dans l'herbe. Oh. Non. Victorina recule les mains. Amir avance trop, d'un pas. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il cherche dans l'herbe, sans se jeter. La pièce a un brin collé. Elle a de l'herbe, papa. Tu la vois, la pièce ? Oui, papa. Il tend la pièce, la main ouverte. Il reste près de l'herbe. Victorina regarde longtemps. Elle prend la pièce. Elle la pose dans le trou. Chien. Chien. Merci, Amir. Maman a vu la main ouverte. Le chien est entier, vous deux ? Oui, papa. Un éclat de table luit sur le bord. L'éclat, maman ? Tu le vois, sur le bois ? Oui, maman.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman aide Victorina à mettre son manteau. Les boutons sont ronds et lisses. Victorina fait un petit signe. À demain ? À demain. Le bateau sèche encore sur le rebord. Et le port reste au parc. Deux eaux, aujourd'hui. La pomme reste dans la poche. Le bateau sèche encore un peu. La tache est partie.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Au parc, une table de bois se tient près de l'herbe. Tu poses le puzzle ici, Amir ? Oui, papa. Maman ouvre le cartable sur l'herbe. Le chat est entier, Amir ? Le chien n'est pas fini. Victorina s'assoit, sans un mot. Je finis, maintenant ! Il pousse la dernière pièce trop vite. La pièce part dans l'herbe. Oh. Non. Victorina recule les mains. Amir avance trop, d'un pas. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il cherche dans l'herbe, sans se jeter. La pièce a un brin collé. Elle a de l'herbe, papa. Tu la vois, la pièce ? Oui, papa. Il tend la pièce, la main ouverte. Il reste près de l'herbe. Victorina regarde longtemps. Elle prend la pièce. Elle la pose dans le trou. Chien. Chien. Merci, Amir. Maman a vu la main ouverte. Le chien est entier, vous deux ? Oui, papa. Un &lt;emphasis level="moderate"&gt;éclat de table&lt;/emphasis&gt; luit sur le bord. L'éclat, maman ? Tu le vois, sur le bois ? Oui, maman.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman aide Iris à mettre son manteau. Iris fait un petit signe. Ruben dit : à de&lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>&lt;low-pitch&gt;Au parc, une table de bois se tient près de l'herbe. Tu poses le puzzle ici, Amir ? Oui, papa. Maman ouvre le cartable sur l'herbe. Le chat est entier, Amir ? Le chien n'est pas fini. Victorina s'assoit, sans un mot. Je finis, maintenant ! Il pousse la dernière pièce trop vite. La pièce part dans l'herbe. Oh. Non. Victorina recule les mains. Amir avance trop, d'un pas. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il cherche dans l'herbe, sans se jeter. La pièce a un brin collé. Elle a de l'herbe, papa. Tu la vois, la pièce ? Oui, papa. Il tend la pièce, la main ouverte. Il reste près de l'herbe. Victorina regarde longtemps. Elle prend la pièce. Elle la pose dans le trou. Chien. Chien. Merci, Amir. Maman a vu la main ouverte. Le chien est entier, vous deux ? Oui, papa. Un &lt;emphasis&gt;éclat de table&lt;/emphasis&gt; luit sur le bord. L'éclat, maman ? Tu le vois, sur le bois ? Oui, maman.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1838,7 +1887,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1846,22 +1895,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1872,30 +1925,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de table</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1904,34 +1957,69 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=2e_ruse_au_parc_il_refuse_de_foncer; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman aide Victorina à mettre son manteau.
-narrateur|Les boutons sont ronds et lisses.
-narrateur|Victorina fait un petit signe.
-papa|À demain ?
-enfant-m|À demain.
-maman|Le bateau sèche encore sur le rebord.
-enfant-m|Et le port reste au parc.
-papa|Deux eaux, aujourd'hui.
-narrateur|La pomme reste dans la poche.
-narrateur|Le bateau sèche encore un peu.
-enfant-m|La tache est partie.</t>
+          <t>narrateur|Au parc, une table de bois se tient près de l'herbe.
+papa|Tu poses le puzzle ici, Amir ?
+enfant-m|Oui, papa.
+narrateur|Maman ouvre le cartable sur l'herbe.
+maman|Le chat est entier, Amir ?
+enfant-m|Le chien n'est pas fini.
+narrateur|Victorina s'assoit, sans un mot.
+enfant-m|Je finis, maintenant !
+narrateur|Il pousse la dernière pièce trop vite.
+narrateur|La pièce part dans l'herbe.
+enfant-m|Oh.
+copine|Non.
+narrateur|Victorina recule les mains.
+narrateur|Amir avance trop, d'un pas.
+narrateur|Amir refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il cherche dans l'herbe, sans se jeter.
+narrateur|La pièce a un brin collé.
+enfant-m|Elle a de l'herbe, papa.
+papa|Tu la vois, la pièce ?
+enfant-m|Oui, papa.
+narrateur|Il tend la pièce, la main ouverte.
+narrateur|Il reste près de l'herbe.
+narrateur|Victorina regarde longtemps.
+narrateur|Elle prend la pièce.
+narrateur|Elle la pose dans le trou.
+copine|Chien.
+enfant-m|Chien.
+maman|Merci, Amir.
+narrateur|Maman a vu la main ouverte.
+papa|Le chien est entier, vous deux ?
+enfant-m|Oui, papa.
+narrateur|Un éclat de table luit sur le bord.
+enfant-m|L'éclat, maman ?
+maman|Tu le vois, sur le bois ?
+enfant-m|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>enfants_parc</t>
         </is>
       </c>
     </row>
@@ -1958,17 +2046,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le bateau a touché l'autre bord. Le port a un quai. Peu de mots, deux voyages.</t>
+          <t>De retour, le crayon jaune est sur le bois. Il n'est plus sous la table. Tu l'as vu, Amir ? Oui, papa. Le puzzle rentre dans le cartable. Le brin d'herbe est resté, Amir ? Sur le chien, maman. Chat. Chat. Le chat a sa tête, vous deux ? Oui, papa. Un carré de soleil tient sur la vitre. La craie, maman. Tu la sens, la craie ? Un peu, maman. Un éclat de table tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le bateau a touché l'autre bord. Le port a un quai. Peu de mots, deux voyages.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;De retour, le crayon jaune est sur le bois. Il n'est plus sous la table. Tu l'as vu, Amir ? Oui, papa. Le puzzle rentre dans le cartable. Le brin d'herbe est resté, Amir ? Sur le chien, maman. Chat. Chat. Le chat a sa tête, vous deux ? Oui, papa. Un carré de soleil tient sur la vitre. La craie, maman. Tu la sens, la craie ? Un peu, maman. Un &lt;emphasis level="moderate"&gt;éclat de table&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;De retour, le crayon jaune est sur le bois. Il n'est plus sous la table. Tu l'as vu, Amir ? Oui, papa. Le puzzle rentre dans le cartable. Le brin d'herbe est resté, Amir ? Sur le chien, maman. Chat. Chat. Le chat a sa tête, vous deux ? Oui, papa. Un carré de soleil tient sur la vitre. La craie, maman. Tu la sens, la craie ? Un peu, maman. Un &lt;emphasis&gt;éclat de table&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2015,15 +2103,15 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2035,12 +2123,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2049,17 +2137,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de table</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2068,11 +2160,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2081,26 +2173,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|Le bateau a touché l'autre bord.
-maman|Le port a un quai.
-papa|Peu de mots, deux voyages.</t>
+          <t>narrateur|De retour, le crayon jaune est sur le bois.
+enfant-m|Il n'est plus sous la table.
+papa|Tu l'as vu, Amir ?
+enfant-m|Oui, papa.
+narrateur|Le puzzle rentre dans le cartable.
+maman|Le brin d'herbe est resté, Amir ?
+enfant-m|Sur le chien, maman.
+copine|Chat.
+enfant-m|Chat.
+papa|Le chat a sa tête, vous deux ?
+enfant-m|Oui, papa.
+narrateur|Un carré de soleil tient sur la vitre.
+enfant-m|La craie, maman.
+maman|Tu la sens, la craie ?
+enfant-m|Un peu, maman.
+narrateur|Un éclat de table tient sur le bois.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>crayon,cartable</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2178,6 +2292,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>